<commit_message>
PROM06: AI quality scoring sheets; TC13-TC15 scans and PR comments
Adds Scoring Rules, AI Quality Scoring (37 independent runs, 0-2 rubric)
and Inter-rater Check sheets to the verified matrix. Archives local
Checkov/tfsec output for TC13-TC15 and PR comments for #82-#84.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019GGG1f33Kz2g4dpPAJoY44
</commit_message>
<xml_diff>
--- a/evidence/prom06/PROM06_TC01-TC12_Verified_Results_Matrix.xlsx
+++ b/evidence/prom06/PROM06_TC01-TC12_Verified_Results_Matrix.xlsx
@@ -15,9 +15,13 @@
     <sheet name="Scanner Results" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Hybrid Runs (Condition C)" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Decisions &amp; Caveats" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="Draft Matrix (original)" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Scoring Rules" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="AI Quality Scoring" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Inter-rater Check" sheetId="10" state="visible" r:id="rId12"/>
+    <sheet name="Draft Matrix (original)" sheetId="11" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="true" localSheetId="8" name="_xlnm._FilterDatabase" vbProcedure="false">'AI Quality Scoring'!$A$1:$R$38</definedName>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Independent AI Runs'!$A$1:$M$38</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Verified Matrix'!$A$1:$O$13</definedName>
   </definedNames>
@@ -31,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1345" uniqueCount="594">
   <si>
     <t xml:space="preserve">PROM06 TC01–TC12 Verified Results Matrix</t>
   </si>
@@ -1262,6 +1266,504 @@
   </si>
   <si>
     <t xml:space="preserve">Close PRs #56–#81 without merging after sign-off</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI explanation and remediation quality — operational scoring rules</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rubric dimensions and 0–2 scale come from the TC01–TC12 Ground-Truth Matrix (remediation-quality rubric). The operational definitions below were written on 13 Oct 2026 to make the rubric applicable consistently. They were written AFTER the AI outputs had been read, by an AI assistant (Claude) acting as scorer; see the disclosure at the bottom.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 = full</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 = partial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 = none / wrong</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D  Detection correctness (vulnerable case)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target condition raised as CONFIRMED on the correct resource.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target raised but as NEEDS_CONTEXT (hidden from PR comment), or only partly identified.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target not raised, classified FALSE_POSITIVE, or run failed validation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D  Detection correctness (non-vulnerable case)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No confirmed finding against the acceptable configuration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only a LOW or unrelated confirmed finding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blocks (fails the gate on) the acceptable configuration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E  Explanation accuracy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every technical and policy claim is correct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contains one or more inaccurate claims, or maps the finding to an inapplicable policy (e.g. SEC-001 'public exposure' applied to IAM, TLS or secrets; tags claimed on a non-taggable resource type).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Core explanation materially wrong.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I  Impact explanation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Specific consequence for this configuration (who can reach/do what).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generic or partly inaccurate impact.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R  Remediation quality</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correct, actionable, addresses the root cause and would yield the ground-truth secure state.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partly correct, or misses part of the secure state, or adds questionable advice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wrong or absent.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C  Context awareness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correctly uses related resources/files (associations, requirements, other files).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Some context used but incomplete or misread.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ignores relevant context.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U  Developer usefulness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A developer could act on the PR comment immediately; no noise.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Useful but with noise: extra false or duplicate CONFIRMED findings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Misleading or useless in the PR comment: target hidden (NEEDS_CONTEXT is not shown), run failed, or legitimate configuration blocked.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Application notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Scope: vulnerable cases (TC02–TC11) are scored on all six dimensions (max 12). Non-vulnerable cases (TC01, TC12) are scored on D, E and U only (max 6); I, R and C are 'n/a'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Each run is scored separately (3 runs per case; 4 for TC08 because one PR run failed validation and a fourth dispatch was made).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Only the AI output of the INDEPENDENT condition is scored (scanner_findings_supplied_to_ai = false). Hybrid (Condition C) outputs are not scored here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Policy mis-mapping is penalised under E only (not U) to avoid double counting; it is also flagged separately in column O of 'AI Quality Scoring' so analysis can exclude it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Disclosure / validity threat: the scorer is an AI assistant that read all outputs before writing these rules. To mitigate, AB should independently score the stratified sample on 'Inter-rater Check' before results are reported; agreement is calculated there.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. TC13–TC15 (added 13 Oct 2026) are not yet scored: their full ai_output.json artefacts still need to be downloaded.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ground truth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target status in AI output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Score %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy mis-map?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noise in PR comment?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scorer justification</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404582550</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not vulnerable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No confirmed findings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n/a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean. One FALSE_POSITIVE informational note (DNS zone name split) correctly dismissed; not shown in PR comment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405003190</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No findings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean; no findings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405111880</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean. Three FALSE_POSITIVE informational notes, all correct dismissals (outbound deny, DDoS not applicable, NSG association present).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404584887</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIRMED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SSH 22 from 0.0.0.0/0 identified on the correct rule; specific internet brute-force impact; restrict source to approved CIDR/Bastion; uses NSG–subnet association.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405012851</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 1; accurate and actionable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405121064</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404589228</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RDP 3389 from any source; SEC-001 mapping appropriate (public exposure); remediation restricts source / Bastion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405022162</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405130215</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target correct, but a second CONFIRMED HIGH finding (F-002 'SEC-001 violation') duplicates F-001 — duplicate noise in the PR comment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404592498</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTP 80 from any source identified; impact framed as generic exposure with no reference to unencrypted HTTP; remediation restricts source only, no HTTPS/redirect alternative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405031009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 1 (no unencrypted-transport reasoning, no HTTPS alternative).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405139458</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404594354</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing subnet–NSG association found by cross-file reasoning (NSG exists, no association). Extra NEEDS_CONTEXT LOW note on DNS comment, not shown in PR comment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405039302</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405149036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 1 (severity MEDIUM rather than HIGH; does not affect rubric).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404596950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public DNS resolver on VNet mapped correctly to NET-002; remediation: Azure-provided or internal DNS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405047995</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405157604</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404600206</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min_tls_version TLS1_0 correctly identified with TLS1_2 remediation. TLS finding mapped to SEC-001 (public exposure) — inapplicable; no encryption policy exists in ai/policy.md. Tag finding (owner, cost-center missing) is correct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405057461</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 1 (SEC-001 mis-mapping; tag finding correct).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405166219</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404605125</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FALSE_POSITIVE (run failed validation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing NSG diagnostic setting raised but classified FALSE_POSITIVE while mapped to LOG-001; validate_review rejected output, run failed. Summary misreads the comment as stating the omission is intentional. Recommendation itself correct. No PR comment produced.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405066857</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NEEDS_CONTEXT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Explanation, impact and remediation (diagnostic setting with both NSG categories) accurate, but NEEDS_CONTEXT is not shown in the PR comment, so the developer sees no finding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405174844</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405218950</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIRMED and mapped to LOG-001 with a complete azurerm_monitor_diagnostic_setting example.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404607277</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hard-coded credential in local found (scanners missed it). Claims the unused local would appear in state/plan — inaccurate for an unreferenced local. Remediation (Key Vault / sensitive variable, rotate) correct.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405075984</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 1, plus mapped to SEC-001 (public exposure) — inapplicable to secrets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405183161</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404612132</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wildcard Actions at subscription scope correctly identified. Second CONFIRMED finding claims azurerm_role_definition needs TAG-001 tags — resource is not taggable (false positive). Remediation includes questionable lifecycle advice.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405084901</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target correct; mapped to SEC-001 (public exposure) — inapplicable to IAM.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405192342</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target correct; SEC-001 mis-mapping plus false TAG-001 finding on non-taggable role definition.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404613836</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wildcard custom role vs documented least-privilege task requirement in another file identified; SEC-001 mis-mapping. (Construct not isolated: wildcard alone also triggers Checkov CKV_AZURE_39.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405093864</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 1; explicitly compares against documented task requirements.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405200842</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As run 2, without policy mis-mapping.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38404619147</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIRMED HIGH (blocks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legitimate public HTTPS treated as HIGH vulnerability; gate blocked (score 50). Also claims azurerm_network_security_rule supports tags (false).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405103514</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFIRMED LOW (tag) only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HTTPS exposure correctly not confirmed (destination-scope note as NEEDS_CONTEXT). Confirmed LOW TAG-001 finding is false: network security rules are not taggable.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">38405210047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Correctly accepted; correctly states rules are not taggable. Caveat: cites the fixture comment 'Ground truth: public TCP/443 ingress is intentional' — the test file cues the answer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blue = scorer input (0–2). Totals and percentages are formulas. Source: ai_output.json in each prom06-INDEPENDENT-&lt;run_id&gt; artefact; rules on 'Scoring Rules'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Summary (formulas)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean — vulnerable runs (TC02–TC11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean — non-vulnerable runs (TC01, TC12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runs with policy mis-mapping</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runs with noise in PR comment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vulnerable runs scoring 2 on every dimension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per test case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean R (vuln.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean score %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min score %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inter-rater check — AB to score independently</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How to use: before looking at the 'AI Quality Scoring' sheet, open each run's ai_output.json (or PR comment) and the ground truth, apply 'Scoring Rules', and type your 0–2 scores in the yellow cells (columns D–I; leave I/R/C blank for TC01/TC12). Agreement updates automatically. Sample: 10 of 37 runs, stratified to include clean, partial, failed and false-positive cases.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example of the expected format (not part of the sample): TC02 run 1 → D 2, E 2, I 2, R 2, C 2, U 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AB: D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AB: E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AB: I</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AB: R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AB: C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AB: U</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI scorer: D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exact matches</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dimensions scored</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Within 1 point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exact agreement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agreement within 1 point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Green = linked from 'AI Quality Scoring'. Discuss and record any disagreement &gt; 1 point before reporting; do not overwrite the original AI-scorer values.</t>
   </si>
   <si>
     <t xml:space="preserve">Ground-truth vulnerability</t>
@@ -1337,11 +1839,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
+    <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1399,8 +1903,22 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1435,6 +1953,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -1487,7 +2011,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="34">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1556,6 +2080,74 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1565,7 +2157,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1617,6 +2209,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFEDEDED"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF0000FF"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1690,6 +2290,10 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
@@ -1940,6 +2544,958 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:R20"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="4" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="11" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="18" t="s">
+        <v>556</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="18"/>
+      <c r="M3" s="18"/>
+      <c r="N3" s="18"/>
+      <c r="O3" s="18"/>
+      <c r="P3" s="18"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="27" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
+        <v>446</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>447</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="D6" s="19" t="s">
+        <v>558</v>
+      </c>
+      <c r="E6" s="19" t="s">
+        <v>559</v>
+      </c>
+      <c r="F6" s="19" t="s">
+        <v>560</v>
+      </c>
+      <c r="G6" s="19" t="s">
+        <v>561</v>
+      </c>
+      <c r="H6" s="19" t="s">
+        <v>562</v>
+      </c>
+      <c r="I6" s="19" t="s">
+        <v>563</v>
+      </c>
+      <c r="J6" s="19" t="s">
+        <v>564</v>
+      </c>
+      <c r="K6" s="19" t="s">
+        <v>451</v>
+      </c>
+      <c r="L6" s="19" t="s">
+        <v>452</v>
+      </c>
+      <c r="M6" s="19" t="s">
+        <v>453</v>
+      </c>
+      <c r="N6" s="19" t="s">
+        <v>454</v>
+      </c>
+      <c r="O6" s="19" t="s">
+        <v>455</v>
+      </c>
+      <c r="P6" s="19" t="s">
+        <v>565</v>
+      </c>
+      <c r="Q6" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="R6" s="19" t="s">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="31" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C5</f>
+        <v>38404584887</v>
+      </c>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
+      <c r="J7" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G5</f>
+        <v>2</v>
+      </c>
+      <c r="K7" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H5</f>
+        <v>2</v>
+      </c>
+      <c r="L7" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!I5</f>
+        <v>2</v>
+      </c>
+      <c r="M7" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!J5</f>
+        <v>2</v>
+      </c>
+      <c r="N7" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!K5</f>
+        <v>2</v>
+      </c>
+      <c r="O7" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L5</f>
+        <v>2</v>
+      </c>
+      <c r="P7" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D7),ISNUMBER(J7)),--(D7=J7),0)+IF(AND(ISNUMBER(E7),ISNUMBER(K7)),--(E7=K7),0)+IF(AND(ISNUMBER(F7),ISNUMBER(L7)),--(F7=L7),0)+IF(AND(ISNUMBER(G7),ISNUMBER(M7)),--(G7=M7),0)+IF(AND(ISNUMBER(H7),ISNUMBER(N7)),--(H7=N7),0)+IF(AND(ISNUMBER(I7),ISNUMBER(O7)),--(I7=O7),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q7" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D7),ISNUMBER(J7))+--AND(ISNUMBER(E7),ISNUMBER(K7))+--AND(ISNUMBER(F7),ISNUMBER(L7))+--AND(ISNUMBER(G7),ISNUMBER(M7))+--AND(ISNUMBER(H7),ISNUMBER(N7))+--AND(ISNUMBER(I7),ISNUMBER(O7))</f>
+        <v>0</v>
+      </c>
+      <c r="R7" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D7),ISNUMBER(J7)),--(ABS(D7-J7)&lt;=1),0)+IF(AND(ISNUMBER(E7),ISNUMBER(K7)),--(ABS(E7-K7)&lt;=1),0)+IF(AND(ISNUMBER(F7),ISNUMBER(L7)),--(ABS(F7-L7)&lt;=1),0)+IF(AND(ISNUMBER(G7),ISNUMBER(M7)),--(ABS(G7-M7)&lt;=1),0)+IF(AND(ISNUMBER(H7),ISNUMBER(N7)),--(ABS(H7-N7)&lt;=1),0)+IF(AND(ISNUMBER(I7),ISNUMBER(O7)),--(ABS(I7-O7)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="31" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C12</f>
+        <v>38405031009</v>
+      </c>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G12</f>
+        <v>2</v>
+      </c>
+      <c r="K8" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H12</f>
+        <v>2</v>
+      </c>
+      <c r="L8" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!I12</f>
+        <v>1</v>
+      </c>
+      <c r="M8" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!J12</f>
+        <v>1</v>
+      </c>
+      <c r="N8" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!K12</f>
+        <v>2</v>
+      </c>
+      <c r="O8" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L12</f>
+        <v>2</v>
+      </c>
+      <c r="P8" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D8),ISNUMBER(J8)),--(D8=J8),0)+IF(AND(ISNUMBER(E8),ISNUMBER(K8)),--(E8=K8),0)+IF(AND(ISNUMBER(F8),ISNUMBER(L8)),--(F8=L8),0)+IF(AND(ISNUMBER(G8),ISNUMBER(M8)),--(G8=M8),0)+IF(AND(ISNUMBER(H8),ISNUMBER(N8)),--(H8=N8),0)+IF(AND(ISNUMBER(I8),ISNUMBER(O8)),--(I8=O8),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q8" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D8),ISNUMBER(J8))+--AND(ISNUMBER(E8),ISNUMBER(K8))+--AND(ISNUMBER(F8),ISNUMBER(L8))+--AND(ISNUMBER(G8),ISNUMBER(M8))+--AND(ISNUMBER(H8),ISNUMBER(N8))+--AND(ISNUMBER(I8),ISNUMBER(O8))</f>
+        <v>0</v>
+      </c>
+      <c r="R8" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D8),ISNUMBER(J8)),--(ABS(D8-J8)&lt;=1),0)+IF(AND(ISNUMBER(E8),ISNUMBER(K8)),--(ABS(E8-K8)&lt;=1),0)+IF(AND(ISNUMBER(F8),ISNUMBER(L8)),--(ABS(F8-L8)&lt;=1),0)+IF(AND(ISNUMBER(G8),ISNUMBER(M8)),--(ABS(G8-M8)&lt;=1),0)+IF(AND(ISNUMBER(H8),ISNUMBER(N8)),--(ABS(H8-N8)&lt;=1),0)+IF(AND(ISNUMBER(I8),ISNUMBER(O8)),--(ABS(I8-O8)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="31" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C20</f>
+        <v>38404600206</v>
+      </c>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
+      <c r="J9" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G20</f>
+        <v>2</v>
+      </c>
+      <c r="K9" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H20</f>
+        <v>1</v>
+      </c>
+      <c r="L9" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!I20</f>
+        <v>2</v>
+      </c>
+      <c r="M9" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!J20</f>
+        <v>2</v>
+      </c>
+      <c r="N9" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!K20</f>
+        <v>2</v>
+      </c>
+      <c r="O9" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L20</f>
+        <v>2</v>
+      </c>
+      <c r="P9" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D9),ISNUMBER(J9)),--(D9=J9),0)+IF(AND(ISNUMBER(E9),ISNUMBER(K9)),--(E9=K9),0)+IF(AND(ISNUMBER(F9),ISNUMBER(L9)),--(F9=L9),0)+IF(AND(ISNUMBER(G9),ISNUMBER(M9)),--(G9=M9),0)+IF(AND(ISNUMBER(H9),ISNUMBER(N9)),--(H9=N9),0)+IF(AND(ISNUMBER(I9),ISNUMBER(O9)),--(I9=O9),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q9" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D9),ISNUMBER(J9))+--AND(ISNUMBER(E9),ISNUMBER(K9))+--AND(ISNUMBER(F9),ISNUMBER(L9))+--AND(ISNUMBER(G9),ISNUMBER(M9))+--AND(ISNUMBER(H9),ISNUMBER(N9))+--AND(ISNUMBER(I9),ISNUMBER(O9))</f>
+        <v>0</v>
+      </c>
+      <c r="R9" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D9),ISNUMBER(J9)),--(ABS(D9-J9)&lt;=1),0)+IF(AND(ISNUMBER(E9),ISNUMBER(K9)),--(ABS(E9-K9)&lt;=1),0)+IF(AND(ISNUMBER(F9),ISNUMBER(L9)),--(ABS(F9-L9)&lt;=1),0)+IF(AND(ISNUMBER(G9),ISNUMBER(M9)),--(ABS(G9-M9)&lt;=1),0)+IF(AND(ISNUMBER(H9),ISNUMBER(N9)),--(ABS(H9-N9)&lt;=1),0)+IF(AND(ISNUMBER(I9),ISNUMBER(O9)),--(ABS(I9-O9)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="B10" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C23</f>
+        <v>38404605125</v>
+      </c>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G23</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H23</f>
+        <v>1</v>
+      </c>
+      <c r="L10" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!I23</f>
+        <v>1</v>
+      </c>
+      <c r="M10" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!J23</f>
+        <v>2</v>
+      </c>
+      <c r="N10" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!K23</f>
+        <v>1</v>
+      </c>
+      <c r="O10" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L23</f>
+        <v>0</v>
+      </c>
+      <c r="P10" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D10),ISNUMBER(J10)),--(D10=J10),0)+IF(AND(ISNUMBER(E10),ISNUMBER(K10)),--(E10=K10),0)+IF(AND(ISNUMBER(F10),ISNUMBER(L10)),--(F10=L10),0)+IF(AND(ISNUMBER(G10),ISNUMBER(M10)),--(G10=M10),0)+IF(AND(ISNUMBER(H10),ISNUMBER(N10)),--(H10=N10),0)+IF(AND(ISNUMBER(I10),ISNUMBER(O10)),--(I10=O10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D10),ISNUMBER(J10))+--AND(ISNUMBER(E10),ISNUMBER(K10))+--AND(ISNUMBER(F10),ISNUMBER(L10))+--AND(ISNUMBER(G10),ISNUMBER(M10))+--AND(ISNUMBER(H10),ISNUMBER(N10))+--AND(ISNUMBER(I10),ISNUMBER(O10))</f>
+        <v>0</v>
+      </c>
+      <c r="R10" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D10),ISNUMBER(J10)),--(ABS(D10-J10)&lt;=1),0)+IF(AND(ISNUMBER(E10),ISNUMBER(K10)),--(ABS(E10-K10)&lt;=1),0)+IF(AND(ISNUMBER(F10),ISNUMBER(L10)),--(ABS(F10-L10)&lt;=1),0)+IF(AND(ISNUMBER(G10),ISNUMBER(M10)),--(ABS(G10-M10)&lt;=1),0)+IF(AND(ISNUMBER(H10),ISNUMBER(N10)),--(ABS(H10-N10)&lt;=1),0)+IF(AND(ISNUMBER(I10),ISNUMBER(O10)),--(ABS(I10-O10)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="31" t="s">
+        <v>99</v>
+      </c>
+      <c r="B11" s="31" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C26</f>
+        <v>38405218950</v>
+      </c>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
+      <c r="J11" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G26</f>
+        <v>2</v>
+      </c>
+      <c r="K11" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H26</f>
+        <v>2</v>
+      </c>
+      <c r="L11" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!I26</f>
+        <v>2</v>
+      </c>
+      <c r="M11" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!J26</f>
+        <v>2</v>
+      </c>
+      <c r="N11" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!K26</f>
+        <v>2</v>
+      </c>
+      <c r="O11" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L26</f>
+        <v>2</v>
+      </c>
+      <c r="P11" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D11),ISNUMBER(J11)),--(D11=J11),0)+IF(AND(ISNUMBER(E11),ISNUMBER(K11)),--(E11=K11),0)+IF(AND(ISNUMBER(F11),ISNUMBER(L11)),--(F11=L11),0)+IF(AND(ISNUMBER(G11),ISNUMBER(M11)),--(G11=M11),0)+IF(AND(ISNUMBER(H11),ISNUMBER(N11)),--(H11=N11),0)+IF(AND(ISNUMBER(I11),ISNUMBER(O11)),--(I11=O11),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D11),ISNUMBER(J11))+--AND(ISNUMBER(E11),ISNUMBER(K11))+--AND(ISNUMBER(F11),ISNUMBER(L11))+--AND(ISNUMBER(G11),ISNUMBER(M11))+--AND(ISNUMBER(H11),ISNUMBER(N11))+--AND(ISNUMBER(I11),ISNUMBER(O11))</f>
+        <v>0</v>
+      </c>
+      <c r="R11" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D11),ISNUMBER(J11)),--(ABS(D11-J11)&lt;=1),0)+IF(AND(ISNUMBER(E11),ISNUMBER(K11)),--(ABS(E11-K11)&lt;=1),0)+IF(AND(ISNUMBER(F11),ISNUMBER(L11)),--(ABS(F11-L11)&lt;=1),0)+IF(AND(ISNUMBER(G11),ISNUMBER(M11)),--(ABS(G11-M11)&lt;=1),0)+IF(AND(ISNUMBER(H11),ISNUMBER(N11)),--(ABS(H11-N11)&lt;=1),0)+IF(AND(ISNUMBER(I11),ISNUMBER(O11)),--(ABS(I11-O11)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="B12" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C28</f>
+        <v>38405075984</v>
+      </c>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G28</f>
+        <v>2</v>
+      </c>
+      <c r="K12" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H28</f>
+        <v>1</v>
+      </c>
+      <c r="L12" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!I28</f>
+        <v>1</v>
+      </c>
+      <c r="M12" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!J28</f>
+        <v>2</v>
+      </c>
+      <c r="N12" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!K28</f>
+        <v>2</v>
+      </c>
+      <c r="O12" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L28</f>
+        <v>2</v>
+      </c>
+      <c r="P12" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D12),ISNUMBER(J12)),--(D12=J12),0)+IF(AND(ISNUMBER(E12),ISNUMBER(K12)),--(E12=K12),0)+IF(AND(ISNUMBER(F12),ISNUMBER(L12)),--(F12=L12),0)+IF(AND(ISNUMBER(G12),ISNUMBER(M12)),--(G12=M12),0)+IF(AND(ISNUMBER(H12),ISNUMBER(N12)),--(H12=N12),0)+IF(AND(ISNUMBER(I12),ISNUMBER(O12)),--(I12=O12),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q12" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D12),ISNUMBER(J12))+--AND(ISNUMBER(E12),ISNUMBER(K12))+--AND(ISNUMBER(F12),ISNUMBER(L12))+--AND(ISNUMBER(G12),ISNUMBER(M12))+--AND(ISNUMBER(H12),ISNUMBER(N12))+--AND(ISNUMBER(I12),ISNUMBER(O12))</f>
+        <v>0</v>
+      </c>
+      <c r="R12" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D12),ISNUMBER(J12)),--(ABS(D12-J12)&lt;=1),0)+IF(AND(ISNUMBER(E12),ISNUMBER(K12)),--(ABS(E12-K12)&lt;=1),0)+IF(AND(ISNUMBER(F12),ISNUMBER(L12)),--(ABS(F12-L12)&lt;=1),0)+IF(AND(ISNUMBER(G12),ISNUMBER(M12)),--(ABS(G12-M12)&lt;=1),0)+IF(AND(ISNUMBER(H12),ISNUMBER(N12)),--(ABS(H12-N12)&lt;=1),0)+IF(AND(ISNUMBER(I12),ISNUMBER(O12)),--(ABS(I12-O12)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="B13" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C30</f>
+        <v>38404612132</v>
+      </c>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G30</f>
+        <v>2</v>
+      </c>
+      <c r="K13" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H30</f>
+        <v>1</v>
+      </c>
+      <c r="L13" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!I30</f>
+        <v>2</v>
+      </c>
+      <c r="M13" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!J30</f>
+        <v>1</v>
+      </c>
+      <c r="N13" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!K30</f>
+        <v>2</v>
+      </c>
+      <c r="O13" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L30</f>
+        <v>1</v>
+      </c>
+      <c r="P13" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D13),ISNUMBER(J13)),--(D13=J13),0)+IF(AND(ISNUMBER(E13),ISNUMBER(K13)),--(E13=K13),0)+IF(AND(ISNUMBER(F13),ISNUMBER(L13)),--(F13=L13),0)+IF(AND(ISNUMBER(G13),ISNUMBER(M13)),--(G13=M13),0)+IF(AND(ISNUMBER(H13),ISNUMBER(N13)),--(H13=N13),0)+IF(AND(ISNUMBER(I13),ISNUMBER(O13)),--(I13=O13),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q13" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D13),ISNUMBER(J13))+--AND(ISNUMBER(E13),ISNUMBER(K13))+--AND(ISNUMBER(F13),ISNUMBER(L13))+--AND(ISNUMBER(G13),ISNUMBER(M13))+--AND(ISNUMBER(H13),ISNUMBER(N13))+--AND(ISNUMBER(I13),ISNUMBER(O13))</f>
+        <v>0</v>
+      </c>
+      <c r="R13" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D13),ISNUMBER(J13)),--(ABS(D13-J13)&lt;=1),0)+IF(AND(ISNUMBER(E13),ISNUMBER(K13)),--(ABS(E13-K13)&lt;=1),0)+IF(AND(ISNUMBER(F13),ISNUMBER(L13)),--(ABS(F13-L13)&lt;=1),0)+IF(AND(ISNUMBER(G13),ISNUMBER(M13)),--(ABS(G13-M13)&lt;=1),0)+IF(AND(ISNUMBER(H13),ISNUMBER(N13)),--(ABS(H13-N13)&lt;=1),0)+IF(AND(ISNUMBER(I13),ISNUMBER(O13)),--(ABS(I13-O13)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="31" t="s">
+        <v>125</v>
+      </c>
+      <c r="B14" s="31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C35</f>
+        <v>38405200842</v>
+      </c>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="32"/>
+      <c r="I14" s="32"/>
+      <c r="J14" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G35</f>
+        <v>2</v>
+      </c>
+      <c r="K14" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H35</f>
+        <v>2</v>
+      </c>
+      <c r="L14" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!I35</f>
+        <v>2</v>
+      </c>
+      <c r="M14" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!J35</f>
+        <v>2</v>
+      </c>
+      <c r="N14" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!K35</f>
+        <v>2</v>
+      </c>
+      <c r="O14" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L35</f>
+        <v>2</v>
+      </c>
+      <c r="P14" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D14),ISNUMBER(J14)),--(D14=J14),0)+IF(AND(ISNUMBER(E14),ISNUMBER(K14)),--(E14=K14),0)+IF(AND(ISNUMBER(F14),ISNUMBER(L14)),--(F14=L14),0)+IF(AND(ISNUMBER(G14),ISNUMBER(M14)),--(G14=M14),0)+IF(AND(ISNUMBER(H14),ISNUMBER(N14)),--(H14=N14),0)+IF(AND(ISNUMBER(I14),ISNUMBER(O14)),--(I14=O14),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D14),ISNUMBER(J14))+--AND(ISNUMBER(E14),ISNUMBER(K14))+--AND(ISNUMBER(F14),ISNUMBER(L14))+--AND(ISNUMBER(G14),ISNUMBER(M14))+--AND(ISNUMBER(H14),ISNUMBER(N14))+--AND(ISNUMBER(I14),ISNUMBER(O14))</f>
+        <v>0</v>
+      </c>
+      <c r="R14" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D14),ISNUMBER(J14)),--(ABS(D14-J14)&lt;=1),0)+IF(AND(ISNUMBER(E14),ISNUMBER(K14)),--(ABS(E14-K14)&lt;=1),0)+IF(AND(ISNUMBER(F14),ISNUMBER(L14)),--(ABS(F14-L14)&lt;=1),0)+IF(AND(ISNUMBER(G14),ISNUMBER(M14)),--(ABS(G14-M14)&lt;=1),0)+IF(AND(ISNUMBER(H14),ISNUMBER(N14)),--(ABS(H14-N14)&lt;=1),0)+IF(AND(ISNUMBER(I14),ISNUMBER(O14)),--(ABS(I14-O14)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="B15" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C36</f>
+        <v>38404619147</v>
+      </c>
+      <c r="D15" s="32"/>
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G36</f>
+        <v>0</v>
+      </c>
+      <c r="K15" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H36</f>
+        <v>1</v>
+      </c>
+      <c r="L15" s="33" t="str">
+        <f aca="false">'AI Quality Scoring'!I36</f>
+        <v>n/a</v>
+      </c>
+      <c r="M15" s="33" t="str">
+        <f aca="false">'AI Quality Scoring'!J36</f>
+        <v>n/a</v>
+      </c>
+      <c r="N15" s="33" t="str">
+        <f aca="false">'AI Quality Scoring'!K36</f>
+        <v>n/a</v>
+      </c>
+      <c r="O15" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L36</f>
+        <v>0</v>
+      </c>
+      <c r="P15" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D15),ISNUMBER(J15)),--(D15=J15),0)+IF(AND(ISNUMBER(E15),ISNUMBER(K15)),--(E15=K15),0)+IF(AND(ISNUMBER(F15),ISNUMBER(L15)),--(F15=L15),0)+IF(AND(ISNUMBER(G15),ISNUMBER(M15)),--(G15=M15),0)+IF(AND(ISNUMBER(H15),ISNUMBER(N15)),--(H15=N15),0)+IF(AND(ISNUMBER(I15),ISNUMBER(O15)),--(I15=O15),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D15),ISNUMBER(J15))+--AND(ISNUMBER(E15),ISNUMBER(K15))+--AND(ISNUMBER(F15),ISNUMBER(L15))+--AND(ISNUMBER(G15),ISNUMBER(M15))+--AND(ISNUMBER(H15),ISNUMBER(N15))+--AND(ISNUMBER(I15),ISNUMBER(O15))</f>
+        <v>0</v>
+      </c>
+      <c r="R15" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D15),ISNUMBER(J15)),--(ABS(D15-J15)&lt;=1),0)+IF(AND(ISNUMBER(E15),ISNUMBER(K15)),--(ABS(E15-K15)&lt;=1),0)+IF(AND(ISNUMBER(F15),ISNUMBER(L15)),--(ABS(F15-L15)&lt;=1),0)+IF(AND(ISNUMBER(G15),ISNUMBER(M15)),--(ABS(G15-M15)&lt;=1),0)+IF(AND(ISNUMBER(H15),ISNUMBER(N15)),--(ABS(H15-N15)&lt;=1),0)+IF(AND(ISNUMBER(I15),ISNUMBER(O15)),--(ABS(I15-O15)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="31" t="s">
+        <v>132</v>
+      </c>
+      <c r="B16" s="31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="31" t="str">
+        <f aca="false">'AI Quality Scoring'!C37</f>
+        <v>38405103514</v>
+      </c>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!G37</f>
+        <v>1</v>
+      </c>
+      <c r="K16" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!H37</f>
+        <v>1</v>
+      </c>
+      <c r="L16" s="33" t="str">
+        <f aca="false">'AI Quality Scoring'!I37</f>
+        <v>n/a</v>
+      </c>
+      <c r="M16" s="33" t="str">
+        <f aca="false">'AI Quality Scoring'!J37</f>
+        <v>n/a</v>
+      </c>
+      <c r="N16" s="33" t="str">
+        <f aca="false">'AI Quality Scoring'!K37</f>
+        <v>n/a</v>
+      </c>
+      <c r="O16" s="33" t="n">
+        <f aca="false">'AI Quality Scoring'!L37</f>
+        <v>1</v>
+      </c>
+      <c r="P16" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D16),ISNUMBER(J16)),--(D16=J16),0)+IF(AND(ISNUMBER(E16),ISNUMBER(K16)),--(E16=K16),0)+IF(AND(ISNUMBER(F16),ISNUMBER(L16)),--(F16=L16),0)+IF(AND(ISNUMBER(G16),ISNUMBER(M16)),--(G16=M16),0)+IF(AND(ISNUMBER(H16),ISNUMBER(N16)),--(H16=N16),0)+IF(AND(ISNUMBER(I16),ISNUMBER(O16)),--(I16=O16),0)</f>
+        <v>0</v>
+      </c>
+      <c r="Q16" s="31" t="n">
+        <f aca="false">--AND(ISNUMBER(D16),ISNUMBER(J16))+--AND(ISNUMBER(E16),ISNUMBER(K16))+--AND(ISNUMBER(F16),ISNUMBER(L16))+--AND(ISNUMBER(G16),ISNUMBER(M16))+--AND(ISNUMBER(H16),ISNUMBER(N16))+--AND(ISNUMBER(I16),ISNUMBER(O16))</f>
+        <v>0</v>
+      </c>
+      <c r="R16" s="31" t="n">
+        <f aca="false">IF(AND(ISNUMBER(D16),ISNUMBER(J16)),--(ABS(D16-J16)&lt;=1),0)+IF(AND(ISNUMBER(E16),ISNUMBER(K16)),--(ABS(E16-K16)&lt;=1),0)+IF(AND(ISNUMBER(F16),ISNUMBER(L16)),--(ABS(F16-L16)&lt;=1),0)+IF(AND(ISNUMBER(G16),ISNUMBER(M16)),--(ABS(G16-M16)&lt;=1),0)+IF(AND(ISNUMBER(H16),ISNUMBER(N16)),--(ABS(H16-N16)&lt;=1),0)+IF(AND(ISNUMBER(I16),ISNUMBER(O16)),--(ABS(I16-O16)&lt;=1),0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
+        <v>568</v>
+      </c>
+      <c r="D18" s="30" t="str">
+        <f aca="false">IF(SUM(Q7:Q16)=0,"not yet scored",SUM(P7:P16)/SUM(Q7:Q16))</f>
+        <v>not yet scored</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
+        <v>569</v>
+      </c>
+      <c r="D19" s="30" t="str">
+        <f aca="false">IF(SUM(Q7:Q16)=0,"not yet scored",SUM(R7:R16)/SUM(Q7:Q16))</f>
+        <v>not yet scored</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="27" t="s">
+        <v>570</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:R3"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="1" width="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>571</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>572</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>573</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>576</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>576</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>577</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>580</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>581</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>583</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>587</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>588</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>585</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>590</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>591</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>584</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>592</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>578</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>579</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>586</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="s">
+        <v>593</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
@@ -5477,239 +7033,208 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="45"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="5" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="17" t="s">
         <v>405</v>
       </c>
-      <c r="C1" s="5" t="s">
+    </row>
+    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="18" t="s">
         <v>406</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="18"/>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
         <v>407</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="B5" s="19" t="s">
         <v>408</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="6" t="s">
+      <c r="C5" s="19" t="s">
         <v>409</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D5" s="19" t="s">
         <v>410</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>410</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" s="6" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
         <v>411</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="B6" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="C6" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="B5" s="6" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
         <v>415</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="B7" s="6" t="s">
         <v>416</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="C7" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D7" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="D6" s="6" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
         <v>419</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="B8" s="6" t="s">
         <v>420</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="B7" s="6" t="s">
+      <c r="C8" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>418</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>419</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>418</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>418</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>99</v>
+    </row>
+    <row r="9" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
+        <v>423</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>412</v>
+        <v>425</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>419</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>108</v>
+        <v>426</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
+        <v>427</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>412</v>
+        <v>429</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>116</v>
+        <v>430</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
+        <v>431</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>117</v>
+        <v>432</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>418</v>
+        <v>433</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>125</v>
+        <v>434</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>435</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>425</v>
+        <v>436</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>418</v>
+        <v>437</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>426</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>413</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>427</v>
-      </c>
+        <v>438</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="22" t="s">
+        <v>440</v>
+      </c>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+    </row>
+    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="22" t="s">
+        <v>441</v>
+      </c>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+    </row>
+    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="22" t="s">
+        <v>442</v>
+      </c>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+    </row>
+    <row r="18" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="22" t="s">
+        <v>443</v>
+      </c>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+    </row>
+    <row r="19" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="22" t="s">
+        <v>444</v>
+      </c>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+    </row>
+    <row r="20" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="22" t="s">
+        <v>445</v>
+      </c>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
     </row>
   </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A2:D3"/>
+    <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
+    <mergeCell ref="A20:D20"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -5718,4 +7243,2832 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:R62"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="7" style="0" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="90"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
+        <v>446</v>
+      </c>
+      <c r="B1" s="19" t="s">
+        <v>447</v>
+      </c>
+      <c r="C1" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>448</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>449</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>450</v>
+      </c>
+      <c r="H1" s="19" t="s">
+        <v>451</v>
+      </c>
+      <c r="I1" s="19" t="s">
+        <v>452</v>
+      </c>
+      <c r="J1" s="19" t="s">
+        <v>453</v>
+      </c>
+      <c r="K1" s="19" t="s">
+        <v>454</v>
+      </c>
+      <c r="L1" s="19" t="s">
+        <v>455</v>
+      </c>
+      <c r="M1" s="19" t="s">
+        <v>456</v>
+      </c>
+      <c r="N1" s="19" t="s">
+        <v>457</v>
+      </c>
+      <c r="O1" s="19" t="s">
+        <v>458</v>
+      </c>
+      <c r="P1" s="19" t="s">
+        <v>459</v>
+      </c>
+      <c r="Q1" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="R1" s="19" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="23" t="s">
+        <v>462</v>
+      </c>
+      <c r="D2" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E2" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="G2" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="J2" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="K2" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="L2" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" s="25" t="n">
+        <f aca="false">SUM(G2:L2)</f>
+        <v>6</v>
+      </c>
+      <c r="N2" s="25" t="n">
+        <f aca="false">IF(E2="Vulnerable",12,6)</f>
+        <v>6</v>
+      </c>
+      <c r="O2" s="26" t="n">
+        <f aca="false">M2/N2</f>
+        <v>1</v>
+      </c>
+      <c r="P2" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q2" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R2" s="6" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>468</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="G3" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="J3" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="K3" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="L3" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" s="25" t="n">
+        <f aca="false">SUM(G3:L3)</f>
+        <v>6</v>
+      </c>
+      <c r="N3" s="25" t="n">
+        <f aca="false">IF(E3="Vulnerable",12,6)</f>
+        <v>6</v>
+      </c>
+      <c r="O3" s="26" t="n">
+        <f aca="false">M3/N3</f>
+        <v>1</v>
+      </c>
+      <c r="P3" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q3" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>471</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="G4" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="J4" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="K4" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="L4" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" s="25" t="n">
+        <f aca="false">SUM(G4:L4)</f>
+        <v>6</v>
+      </c>
+      <c r="N4" s="25" t="n">
+        <f aca="false">IF(E4="Vulnerable",12,6)</f>
+        <v>6</v>
+      </c>
+      <c r="O4" s="26" t="n">
+        <f aca="false">M4/N4</f>
+        <v>1</v>
+      </c>
+      <c r="P4" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q4" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R4" s="6" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>473</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" s="25" t="n">
+        <f aca="false">SUM(G5:L5)</f>
+        <v>12</v>
+      </c>
+      <c r="N5" s="25" t="n">
+        <f aca="false">IF(E5="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O5" s="26" t="n">
+        <f aca="false">M5/N5</f>
+        <v>1</v>
+      </c>
+      <c r="P5" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q5" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>476</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M6" s="25" t="n">
+        <f aca="false">SUM(G6:L6)</f>
+        <v>12</v>
+      </c>
+      <c r="N6" s="25" t="n">
+        <f aca="false">IF(E6="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O6" s="26" t="n">
+        <f aca="false">M6/N6</f>
+        <v>1</v>
+      </c>
+      <c r="P6" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q6" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>478</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="25" t="n">
+        <f aca="false">SUM(G7:L7)</f>
+        <v>12</v>
+      </c>
+      <c r="N7" s="25" t="n">
+        <f aca="false">IF(E7="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O7" s="26" t="n">
+        <f aca="false">M7/N7</f>
+        <v>1</v>
+      </c>
+      <c r="P7" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q7" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>479</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L8" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" s="25" t="n">
+        <f aca="false">SUM(G8:L8)</f>
+        <v>12</v>
+      </c>
+      <c r="N8" s="25" t="n">
+        <f aca="false">IF(E8="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O8" s="26" t="n">
+        <f aca="false">M8/N8</f>
+        <v>1</v>
+      </c>
+      <c r="P8" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q8" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R8" s="6" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>481</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G9" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H9" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J9" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L9" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="25" t="n">
+        <f aca="false">SUM(G9:L9)</f>
+        <v>12</v>
+      </c>
+      <c r="N9" s="25" t="n">
+        <f aca="false">IF(E9="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O9" s="26" t="n">
+        <f aca="false">M9/N9</f>
+        <v>1</v>
+      </c>
+      <c r="P9" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q9" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>483</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G10" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" s="25" t="n">
+        <f aca="false">SUM(G10:L10)</f>
+        <v>11</v>
+      </c>
+      <c r="N10" s="25" t="n">
+        <f aca="false">IF(E10="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O10" s="26" t="n">
+        <f aca="false">M10/N10</f>
+        <v>0.916666666666667</v>
+      </c>
+      <c r="P10" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q10" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="R10" s="6" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>486</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G11" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L11" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="25" t="n">
+        <f aca="false">SUM(G11:L11)</f>
+        <v>10</v>
+      </c>
+      <c r="N11" s="25" t="n">
+        <f aca="false">IF(E11="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O11" s="26" t="n">
+        <f aca="false">M11/N11</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="P11" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q11" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R11" s="6" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>488</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" s="25" t="n">
+        <f aca="false">SUM(G12:L12)</f>
+        <v>10</v>
+      </c>
+      <c r="N12" s="25" t="n">
+        <f aca="false">IF(E12="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O12" s="26" t="n">
+        <f aca="false">M12/N12</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="P12" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q12" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R12" s="6" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>490</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L13" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M13" s="25" t="n">
+        <f aca="false">SUM(G13:L13)</f>
+        <v>10</v>
+      </c>
+      <c r="N13" s="25" t="n">
+        <f aca="false">IF(E13="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O13" s="26" t="n">
+        <f aca="false">M13/N13</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="P13" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q13" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R13" s="6" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B14" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>491</v>
+      </c>
+      <c r="D14" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L14" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M14" s="25" t="n">
+        <f aca="false">SUM(G14:L14)</f>
+        <v>12</v>
+      </c>
+      <c r="N14" s="25" t="n">
+        <f aca="false">IF(E14="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O14" s="26" t="n">
+        <f aca="false">M14/N14</f>
+        <v>1</v>
+      </c>
+      <c r="P14" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q14" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="23" t="s">
+        <v>493</v>
+      </c>
+      <c r="D15" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E15" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L15" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" s="25" t="n">
+        <f aca="false">SUM(G15:L15)</f>
+        <v>12</v>
+      </c>
+      <c r="N15" s="25" t="n">
+        <f aca="false">IF(E15="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O15" s="26" t="n">
+        <f aca="false">M15/N15</f>
+        <v>1</v>
+      </c>
+      <c r="P15" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q15" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R15" s="6" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="23" t="s">
+        <v>494</v>
+      </c>
+      <c r="D16" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E16" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G16" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J16" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M16" s="25" t="n">
+        <f aca="false">SUM(G16:L16)</f>
+        <v>12</v>
+      </c>
+      <c r="N16" s="25" t="n">
+        <f aca="false">IF(E16="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O16" s="26" t="n">
+        <f aca="false">M16/N16</f>
+        <v>1</v>
+      </c>
+      <c r="P16" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q16" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R16" s="6" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="23" t="s">
+        <v>496</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E17" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G17" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L17" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M17" s="25" t="n">
+        <f aca="false">SUM(G17:L17)</f>
+        <v>12</v>
+      </c>
+      <c r="N17" s="25" t="n">
+        <f aca="false">IF(E17="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O17" s="26" t="n">
+        <f aca="false">M17/N17</f>
+        <v>1</v>
+      </c>
+      <c r="P17" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q17" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R17" s="6" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B18" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>498</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E18" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G18" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K18" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M18" s="25" t="n">
+        <f aca="false">SUM(G18:L18)</f>
+        <v>12</v>
+      </c>
+      <c r="N18" s="25" t="n">
+        <f aca="false">IF(E18="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O18" s="26" t="n">
+        <f aca="false">M18/N18</f>
+        <v>1</v>
+      </c>
+      <c r="P18" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q18" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R18" s="6" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="23" t="s">
+        <v>499</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E19" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M19" s="25" t="n">
+        <f aca="false">SUM(G19:L19)</f>
+        <v>12</v>
+      </c>
+      <c r="N19" s="25" t="n">
+        <f aca="false">IF(E19="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O19" s="26" t="n">
+        <f aca="false">M19/N19</f>
+        <v>1</v>
+      </c>
+      <c r="P19" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q19" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R19" s="6" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="23" t="s">
+        <v>500</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E20" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H20" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L20" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M20" s="25" t="n">
+        <f aca="false">SUM(G20:L20)</f>
+        <v>11</v>
+      </c>
+      <c r="N20" s="25" t="n">
+        <f aca="false">IF(E20="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O20" s="26" t="n">
+        <f aca="false">M20/N20</f>
+        <v>0.916666666666667</v>
+      </c>
+      <c r="P20" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q20" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R20" s="6" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="23" t="s">
+        <v>502</v>
+      </c>
+      <c r="D21" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E21" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H21" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J21" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K21" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L21" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M21" s="25" t="n">
+        <f aca="false">SUM(G21:L21)</f>
+        <v>11</v>
+      </c>
+      <c r="N21" s="25" t="n">
+        <f aca="false">IF(E21="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O21" s="26" t="n">
+        <f aca="false">M21/N21</f>
+        <v>0.916666666666667</v>
+      </c>
+      <c r="P21" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q21" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R21" s="6" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="B22" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>504</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E22" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H22" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L22" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M22" s="25" t="n">
+        <f aca="false">SUM(G22:L22)</f>
+        <v>11</v>
+      </c>
+      <c r="N22" s="25" t="n">
+        <f aca="false">IF(E22="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O22" s="26" t="n">
+        <f aca="false">M22/N22</f>
+        <v>0.916666666666667</v>
+      </c>
+      <c r="P22" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q22" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R22" s="6" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="B23" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>505</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E23" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>506</v>
+      </c>
+      <c r="G23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I23" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="L23" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="25" t="n">
+        <f aca="false">SUM(G23:L23)</f>
+        <v>5</v>
+      </c>
+      <c r="N23" s="25" t="n">
+        <f aca="false">IF(E23="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O23" s="26" t="n">
+        <f aca="false">M23/N23</f>
+        <v>0.416666666666667</v>
+      </c>
+      <c r="P23" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q23" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R23" s="6" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="B24" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>508</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E24" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="G24" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I24" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L24" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="25" t="n">
+        <f aca="false">SUM(G24:L24)</f>
+        <v>9</v>
+      </c>
+      <c r="N24" s="25" t="n">
+        <f aca="false">IF(E24="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O24" s="26" t="n">
+        <f aca="false">M24/N24</f>
+        <v>0.75</v>
+      </c>
+      <c r="P24" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q24" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R24" s="6" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>511</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>509</v>
+      </c>
+      <c r="G25" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I25" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J25" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L25" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="25" t="n">
+        <f aca="false">SUM(G25:L25)</f>
+        <v>9</v>
+      </c>
+      <c r="N25" s="25" t="n">
+        <f aca="false">IF(E25="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O25" s="26" t="n">
+        <f aca="false">M25/N25</f>
+        <v>0.75</v>
+      </c>
+      <c r="P25" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q25" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R25" s="6" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="23" t="s">
+        <v>99</v>
+      </c>
+      <c r="B26" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="23" t="s">
+        <v>513</v>
+      </c>
+      <c r="D26" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E26" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L26" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" s="25" t="n">
+        <f aca="false">SUM(G26:L26)</f>
+        <v>12</v>
+      </c>
+      <c r="N26" s="25" t="n">
+        <f aca="false">IF(E26="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O26" s="26" t="n">
+        <f aca="false">M26/N26</f>
+        <v>1</v>
+      </c>
+      <c r="P26" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q26" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R26" s="6" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="B27" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C27" s="23" t="s">
+        <v>515</v>
+      </c>
+      <c r="D27" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E27" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G27" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H27" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K27" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L27" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" s="25" t="n">
+        <f aca="false">SUM(G27:L27)</f>
+        <v>10</v>
+      </c>
+      <c r="N27" s="25" t="n">
+        <f aca="false">IF(E27="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O27" s="26" t="n">
+        <f aca="false">M27/N27</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="P27" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q27" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R27" s="6" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="B28" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" s="23" t="s">
+        <v>517</v>
+      </c>
+      <c r="D28" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E28" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G28" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L28" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" s="25" t="n">
+        <f aca="false">SUM(G28:L28)</f>
+        <v>10</v>
+      </c>
+      <c r="N28" s="25" t="n">
+        <f aca="false">IF(E28="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O28" s="26" t="n">
+        <f aca="false">M28/N28</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="P28" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q28" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R28" s="6" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="23" t="s">
+        <v>108</v>
+      </c>
+      <c r="B29" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>519</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E29" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G29" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L29" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M29" s="25" t="n">
+        <f aca="false">SUM(G29:L29)</f>
+        <v>10</v>
+      </c>
+      <c r="N29" s="25" t="n">
+        <f aca="false">IF(E29="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O29" s="26" t="n">
+        <f aca="false">M29/N29</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="P29" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q29" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R29" s="6" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B30" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="23" t="s">
+        <v>520</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E30" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G30" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H30" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I30" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J30" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L30" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M30" s="25" t="n">
+        <f aca="false">SUM(G30:L30)</f>
+        <v>9</v>
+      </c>
+      <c r="N30" s="25" t="n">
+        <f aca="false">IF(E30="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O30" s="26" t="n">
+        <f aca="false">M30/N30</f>
+        <v>0.75</v>
+      </c>
+      <c r="P30" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q30" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="R30" s="6" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B31" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>522</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E31" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M31" s="25" t="n">
+        <f aca="false">SUM(G31:L31)</f>
+        <v>11</v>
+      </c>
+      <c r="N31" s="25" t="n">
+        <f aca="false">IF(E31="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O31" s="26" t="n">
+        <f aca="false">M31/N31</f>
+        <v>0.916666666666667</v>
+      </c>
+      <c r="P31" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q31" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R31" s="6" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="23" t="s">
+        <v>116</v>
+      </c>
+      <c r="B32" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" s="23" t="s">
+        <v>524</v>
+      </c>
+      <c r="D32" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E32" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J32" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M32" s="25" t="n">
+        <f aca="false">SUM(G32:L32)</f>
+        <v>10</v>
+      </c>
+      <c r="N32" s="25" t="n">
+        <f aca="false">IF(E32="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O32" s="26" t="n">
+        <f aca="false">M32/N32</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="P32" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q32" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="R32" s="6" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B33" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="23" t="s">
+        <v>526</v>
+      </c>
+      <c r="D33" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E33" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" s="25" t="n">
+        <f aca="false">SUM(G33:L33)</f>
+        <v>11</v>
+      </c>
+      <c r="N33" s="25" t="n">
+        <f aca="false">IF(E33="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O33" s="26" t="n">
+        <f aca="false">M33/N33</f>
+        <v>0.916666666666667</v>
+      </c>
+      <c r="P33" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q33" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R33" s="6" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B34" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" s="23" t="s">
+        <v>528</v>
+      </c>
+      <c r="D34" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E34" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G34" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J34" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K34" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L34" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M34" s="25" t="n">
+        <f aca="false">SUM(G34:L34)</f>
+        <v>11</v>
+      </c>
+      <c r="N34" s="25" t="n">
+        <f aca="false">IF(E34="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O34" s="26" t="n">
+        <f aca="false">M34/N34</f>
+        <v>0.916666666666667</v>
+      </c>
+      <c r="P34" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="Q34" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R34" s="6" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B35" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" s="23" t="s">
+        <v>530</v>
+      </c>
+      <c r="D35" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E35" s="23" t="s">
+        <v>41</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="G35" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H35" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I35" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="J35" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K35" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="L35" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M35" s="25" t="n">
+        <f aca="false">SUM(G35:L35)</f>
+        <v>12</v>
+      </c>
+      <c r="N35" s="25" t="n">
+        <f aca="false">IF(E35="Vulnerable",12,6)</f>
+        <v>12</v>
+      </c>
+      <c r="O35" s="26" t="n">
+        <f aca="false">M35/N35</f>
+        <v>1</v>
+      </c>
+      <c r="P35" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q35" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R35" s="6" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B36" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" s="23" t="s">
+        <v>532</v>
+      </c>
+      <c r="D36" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="E36" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>533</v>
+      </c>
+      <c r="G36" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="J36" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="K36" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="L36" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" s="25" t="n">
+        <f aca="false">SUM(G36:L36)</f>
+        <v>1</v>
+      </c>
+      <c r="N36" s="25" t="n">
+        <f aca="false">IF(E36="Vulnerable",12,6)</f>
+        <v>6</v>
+      </c>
+      <c r="O36" s="26" t="n">
+        <f aca="false">M36/N36</f>
+        <v>0.166666666666667</v>
+      </c>
+      <c r="P36" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q36" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="R36" s="6" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B37" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C37" s="23" t="s">
+        <v>535</v>
+      </c>
+      <c r="D37" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E37" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>536</v>
+      </c>
+      <c r="G37" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="J37" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="K37" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="L37" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="M37" s="25" t="n">
+        <f aca="false">SUM(G37:L37)</f>
+        <v>3</v>
+      </c>
+      <c r="N37" s="25" t="n">
+        <f aca="false">IF(E37="Vulnerable",12,6)</f>
+        <v>6</v>
+      </c>
+      <c r="O37" s="26" t="n">
+        <f aca="false">M37/N37</f>
+        <v>0.5</v>
+      </c>
+      <c r="P37" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q37" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="R37" s="6" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B38" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" s="23" t="s">
+        <v>538</v>
+      </c>
+      <c r="D38" s="23" t="s">
+        <v>197</v>
+      </c>
+      <c r="E38" s="23" t="s">
+        <v>463</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>464</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H38" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="I38" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="J38" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="K38" s="24" t="s">
+        <v>465</v>
+      </c>
+      <c r="L38" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="M38" s="25" t="n">
+        <f aca="false">SUM(G38:L38)</f>
+        <v>6</v>
+      </c>
+      <c r="N38" s="25" t="n">
+        <f aca="false">IF(E38="Vulnerable",12,6)</f>
+        <v>6</v>
+      </c>
+      <c r="O38" s="26" t="n">
+        <f aca="false">M38/N38</f>
+        <v>1</v>
+      </c>
+      <c r="P38" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="Q38" s="25" t="s">
+        <v>466</v>
+      </c>
+      <c r="R38" s="6" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="27" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="17" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="28" t="s">
+        <v>145</v>
+      </c>
+      <c r="G42" s="28" t="s">
+        <v>450</v>
+      </c>
+      <c r="H42" s="28" t="s">
+        <v>451</v>
+      </c>
+      <c r="I42" s="28" t="s">
+        <v>452</v>
+      </c>
+      <c r="J42" s="28" t="s">
+        <v>453</v>
+      </c>
+      <c r="K42" s="28" t="s">
+        <v>454</v>
+      </c>
+      <c r="L42" s="28" t="s">
+        <v>455</v>
+      </c>
+      <c r="O42" s="28" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="21" t="s">
+        <v>542</v>
+      </c>
+      <c r="G43" s="29" t="n">
+        <f aca="false">AVERAGEIFS(G$2:G$38,$E$2:$E$38,"Vulnerable")</f>
+        <v>1.87096774193548</v>
+      </c>
+      <c r="H43" s="29" t="n">
+        <f aca="false">AVERAGEIFS(H$2:H$38,$E$2:$E$38,"Vulnerable")</f>
+        <v>1.61290322580645</v>
+      </c>
+      <c r="I43" s="29" t="n">
+        <f aca="false">AVERAGEIFS(I$2:I$38,$E$2:$E$38,"Vulnerable")</f>
+        <v>1.7741935483871</v>
+      </c>
+      <c r="J43" s="29" t="n">
+        <f aca="false">AVERAGEIFS(J$2:J$38,$E$2:$E$38,"Vulnerable")</f>
+        <v>1.87096774193548</v>
+      </c>
+      <c r="K43" s="29" t="n">
+        <f aca="false">AVERAGEIFS(K$2:K$38,$E$2:$E$38,"Vulnerable")</f>
+        <v>1.96774193548387</v>
+      </c>
+      <c r="L43" s="29" t="n">
+        <f aca="false">AVERAGEIFS(L$2:L$38,$E$2:$E$38,"Vulnerable")</f>
+        <v>1.70967741935484</v>
+      </c>
+      <c r="O43" s="30" t="n">
+        <f aca="false">AVERAGEIFS(O$2:O$38,$E$2:$E$38,"Vulnerable")</f>
+        <v>0.900537634408602</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21" t="s">
+        <v>543</v>
+      </c>
+      <c r="G44" s="29" t="n">
+        <f aca="false">AVERAGEIFS(G$2:G$38,$E$2:$E$38,"Not vulnerable")</f>
+        <v>1.5</v>
+      </c>
+      <c r="H44" s="29" t="n">
+        <f aca="false">AVERAGEIFS(H$2:H$38,$E$2:$E$38,"Not vulnerable")</f>
+        <v>1.66666666666667</v>
+      </c>
+      <c r="I44" s="0" t="s">
+        <v>465</v>
+      </c>
+      <c r="J44" s="0" t="s">
+        <v>465</v>
+      </c>
+      <c r="K44" s="0" t="s">
+        <v>465</v>
+      </c>
+      <c r="L44" s="29" t="n">
+        <f aca="false">AVERAGEIFS(L$2:L$38,$E$2:$E$38,"Not vulnerable")</f>
+        <v>1.5</v>
+      </c>
+      <c r="O44" s="30" t="n">
+        <f aca="false">AVERAGEIFS(O$2:O$38,$E$2:$E$38,"Not vulnerable")</f>
+        <v>0.777777777777778</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21" t="s">
+        <v>544</v>
+      </c>
+      <c r="G45" s="0" t="str">
+        <f aca="false">COUNTIF(P$2:P$38,"Y")&amp;" of "&amp;COUNTA(P$2:P$38)</f>
+        <v>9 of 37</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21" t="s">
+        <v>545</v>
+      </c>
+      <c r="G46" s="0" t="str">
+        <f aca="false">COUNTIF(Q$2:Q$38,"Y")&amp;" of "&amp;COUNTA(Q$2:Q$38)</f>
+        <v>5 of 37</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="21" t="s">
+        <v>546</v>
+      </c>
+      <c r="G47" s="0" t="str">
+        <f aca="false">SUMPRODUCT(($E$2:$E$38="Vulnerable")*(M$2:M$38=12))&amp;" of "&amp;COUNTIF($E$2:$E$38,"Vulnerable")</f>
+        <v>13 of 31</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="17" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="28" t="s">
+        <v>446</v>
+      </c>
+      <c r="B50" s="28" t="s">
+        <v>548</v>
+      </c>
+      <c r="C50" s="28" t="s">
+        <v>549</v>
+      </c>
+      <c r="D50" s="28" t="s">
+        <v>550</v>
+      </c>
+      <c r="E50" s="28" t="s">
+        <v>551</v>
+      </c>
+      <c r="F50" s="28" t="s">
+        <v>552</v>
+      </c>
+      <c r="G50" s="28" t="s">
+        <v>553</v>
+      </c>
+      <c r="H50" s="28" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B51" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A51)</f>
+        <v>3</v>
+      </c>
+      <c r="C51" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A51,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D51" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A51,H$2:H$38)</f>
+        <v>2</v>
+      </c>
+      <c r="E51" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A51,L$2:L$38)</f>
+        <v>2</v>
+      </c>
+      <c r="F51" s="29" t="str">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A51,J$2:J$38),"n/a")</f>
+        <v>n/a</v>
+      </c>
+      <c r="G51" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A51,O$2:O$38)</f>
+        <v>1</v>
+      </c>
+      <c r="H51" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A51)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B52" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A52)</f>
+        <v>3</v>
+      </c>
+      <c r="C52" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A52,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D52" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A52,H$2:H$38)</f>
+        <v>2</v>
+      </c>
+      <c r="E52" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A52,L$2:L$38)</f>
+        <v>2</v>
+      </c>
+      <c r="F52" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A52,J$2:J$38),"n/a")</f>
+        <v>2</v>
+      </c>
+      <c r="G52" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A52,O$2:O$38)</f>
+        <v>1</v>
+      </c>
+      <c r="H52" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A52)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="B53" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A53)</f>
+        <v>3</v>
+      </c>
+      <c r="C53" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A53,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D53" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A53,H$2:H$38)</f>
+        <v>2</v>
+      </c>
+      <c r="E53" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A53,L$2:L$38)</f>
+        <v>1.66666666666667</v>
+      </c>
+      <c r="F53" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A53,J$2:J$38),"n/a")</f>
+        <v>2</v>
+      </c>
+      <c r="G53" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A53,O$2:O$38)</f>
+        <v>0.972222222222222</v>
+      </c>
+      <c r="H53" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A53)</f>
+        <v>0.916666666666667</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="B54" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A54)</f>
+        <v>3</v>
+      </c>
+      <c r="C54" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A54,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D54" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A54,H$2:H$38)</f>
+        <v>2</v>
+      </c>
+      <c r="E54" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A54,L$2:L$38)</f>
+        <v>2</v>
+      </c>
+      <c r="F54" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A54,J$2:J$38),"n/a")</f>
+        <v>1</v>
+      </c>
+      <c r="G54" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A54,O$2:O$38)</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="H54" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A54)</f>
+        <v>0.833333333333333</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="B55" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A55)</f>
+        <v>3</v>
+      </c>
+      <c r="C55" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A55,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D55" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A55,H$2:H$38)</f>
+        <v>2</v>
+      </c>
+      <c r="E55" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A55,L$2:L$38)</f>
+        <v>2</v>
+      </c>
+      <c r="F55" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A55,J$2:J$38),"n/a")</f>
+        <v>2</v>
+      </c>
+      <c r="G55" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A55,O$2:O$38)</f>
+        <v>1</v>
+      </c>
+      <c r="H55" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A55)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="B56" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A56)</f>
+        <v>3</v>
+      </c>
+      <c r="C56" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A56,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D56" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A56,H$2:H$38)</f>
+        <v>2</v>
+      </c>
+      <c r="E56" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A56,L$2:L$38)</f>
+        <v>2</v>
+      </c>
+      <c r="F56" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A56,J$2:J$38),"n/a")</f>
+        <v>2</v>
+      </c>
+      <c r="G56" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A56,O$2:O$38)</f>
+        <v>1</v>
+      </c>
+      <c r="H56" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A56)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B57" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A57)</f>
+        <v>3</v>
+      </c>
+      <c r="C57" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A57,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D57" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A57,H$2:H$38)</f>
+        <v>1</v>
+      </c>
+      <c r="E57" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A57,L$2:L$38)</f>
+        <v>2</v>
+      </c>
+      <c r="F57" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A57,J$2:J$38),"n/a")</f>
+        <v>2</v>
+      </c>
+      <c r="G57" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A57,O$2:O$38)</f>
+        <v>0.916666666666667</v>
+      </c>
+      <c r="H57" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A57)</f>
+        <v>0.916666666666667</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="B58" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A58)</f>
+        <v>4</v>
+      </c>
+      <c r="C58" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A58,G$2:G$38)</f>
+        <v>1</v>
+      </c>
+      <c r="D58" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A58,H$2:H$38)</f>
+        <v>1.75</v>
+      </c>
+      <c r="E58" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A58,L$2:L$38)</f>
+        <v>0.5</v>
+      </c>
+      <c r="F58" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A58,J$2:J$38),"n/a")</f>
+        <v>2</v>
+      </c>
+      <c r="G58" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A58,O$2:O$38)</f>
+        <v>0.729166666666667</v>
+      </c>
+      <c r="H58" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A58)</f>
+        <v>0.416666666666667</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="B59" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A59)</f>
+        <v>3</v>
+      </c>
+      <c r="C59" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A59,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D59" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A59,H$2:H$38)</f>
+        <v>1</v>
+      </c>
+      <c r="E59" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A59,L$2:L$38)</f>
+        <v>2</v>
+      </c>
+      <c r="F59" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A59,J$2:J$38),"n/a")</f>
+        <v>2</v>
+      </c>
+      <c r="G59" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A59,O$2:O$38)</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="H59" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A59)</f>
+        <v>0.833333333333333</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="B60" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A60)</f>
+        <v>3</v>
+      </c>
+      <c r="C60" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A60,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D60" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A60,H$2:H$38)</f>
+        <v>1</v>
+      </c>
+      <c r="E60" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A60,L$2:L$38)</f>
+        <v>1.33333333333333</v>
+      </c>
+      <c r="F60" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A60,J$2:J$38),"n/a")</f>
+        <v>1.66666666666667</v>
+      </c>
+      <c r="G60" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A60,O$2:O$38)</f>
+        <v>0.833333333333333</v>
+      </c>
+      <c r="H60" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A60)</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="B61" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A61)</f>
+        <v>3</v>
+      </c>
+      <c r="C61" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A61,G$2:G$38)</f>
+        <v>2</v>
+      </c>
+      <c r="D61" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A61,H$2:H$38)</f>
+        <v>1.33333333333333</v>
+      </c>
+      <c r="E61" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A61,L$2:L$38)</f>
+        <v>2</v>
+      </c>
+      <c r="F61" s="29" t="n">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A61,J$2:J$38),"n/a")</f>
+        <v>2</v>
+      </c>
+      <c r="G61" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A61,O$2:O$38)</f>
+        <v>0.944444444444444</v>
+      </c>
+      <c r="H61" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A61)</f>
+        <v>0.916666666666667</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="B62" s="0" t="n">
+        <f aca="false">COUNTIF($A$2:$A$38,A62)</f>
+        <v>3</v>
+      </c>
+      <c r="C62" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A62,G$2:G$38)</f>
+        <v>1</v>
+      </c>
+      <c r="D62" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A62,H$2:H$38)</f>
+        <v>1.33333333333333</v>
+      </c>
+      <c r="E62" s="29" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A62,L$2:L$38)</f>
+        <v>1</v>
+      </c>
+      <c r="F62" s="29" t="str">
+        <f aca="false">IFERROR(AVERAGEIF($A$2:$A$38,A62,J$2:J$38),"n/a")</f>
+        <v>n/a</v>
+      </c>
+      <c r="G62" s="30" t="n">
+        <f aca="false">AVERAGEIF($A$2:$A$38,A62,O$2:O$38)</f>
+        <v>0.555555555555556</v>
+      </c>
+      <c r="H62" s="30" t="n">
+        <f aca="false">_xlfn.MINIFS(O$2:O$38,$A$2:$A$38,A62)</f>
+        <v>0.166666666666667</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:R38"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>